<commit_message>
Actualizar analisis automatico ARQ v2
</commit_message>
<xml_diff>
--- a/historial_senales.xlsx
+++ b/historial_senales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,36 +551,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-13-SMCI</t>
+          <t>2026-05-14-ZS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Servidores IA</t>
+          <t>Ciberseguridad</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>POSIBLE COMPRA</t>
+          <t>COMPRA FUERTE</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>BUY STRONG</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -588,22 +588,22 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>32.21</v>
+        <v>152.43</v>
       </c>
       <c r="J2" t="n">
-        <v>32</v>
+        <v>152.43</v>
       </c>
       <c r="K2" t="n">
-        <v>31.41</v>
+        <v>150.02</v>
       </c>
       <c r="L2" t="n">
-        <v>32.55</v>
+        <v>153.46</v>
       </c>
       <c r="M2" t="n">
-        <v>29.11</v>
+        <v>143.12</v>
       </c>
       <c r="N2" t="n">
-        <v>37.26</v>
+        <v>167.6</v>
       </c>
       <c r="O2" t="n">
         <v>1.63</v>
@@ -619,30 +619,30 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>-0.65</v>
+        <v>0</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
         <v>0</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.65</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>POSIBLE COMPRA</t>
+          <t>COMPRA FUERTE</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>BUY STRONG</t>
         </is>
       </c>
       <c r="Y2" t="n">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -653,22 +653,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-13-NVDA</t>
+          <t>2026-05-14-XLV</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>IA / Chips</t>
+          <t>ETF Salud</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -682,30 +682,30 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>226.34</v>
+        <v>146.71</v>
       </c>
       <c r="J3" t="n">
-        <v>225.83</v>
+        <v>146.71</v>
       </c>
       <c r="K3" t="n">
-        <v>223.5</v>
+        <v>146.03</v>
       </c>
       <c r="L3" t="n">
-        <v>227.56</v>
+        <v>147</v>
       </c>
       <c r="M3" t="n">
-        <v>215.39</v>
+        <v>144.07</v>
       </c>
       <c r="N3" t="n">
-        <v>244.18</v>
+        <v>151.01</v>
       </c>
       <c r="O3" t="n">
         <v>1.63</v>
@@ -721,14 +721,14 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>-0.23</v>
+        <v>0</v>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.23</v>
+        <v>0</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -744,33 +744,33 @@
         </is>
       </c>
       <c r="Y3" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-12-XOM</t>
+          <t>2026-05-14-XLE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Energía</t>
+          <t>ETF Energía</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -792,22 +792,22 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>150.85</v>
+        <v>57.63</v>
       </c>
       <c r="J4" t="n">
-        <v>151.57</v>
+        <v>57.63</v>
       </c>
       <c r="K4" t="n">
-        <v>149.44</v>
+        <v>57.17</v>
       </c>
       <c r="L4" t="n">
-        <v>151.45</v>
+        <v>57.83</v>
       </c>
       <c r="M4" t="n">
-        <v>145.42</v>
+        <v>55.85</v>
       </c>
       <c r="N4" t="n">
-        <v>159.7</v>
+        <v>60.54</v>
       </c>
       <c r="O4" t="n">
         <v>1.63</v>
@@ -823,17 +823,17 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.15</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="Y4" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -857,22 +857,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-12-TSM</t>
+          <t>2026-05-14-WMT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Chips</t>
+          <t>Consumo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -894,22 +894,22 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>392.55</v>
+        <v>131.47</v>
       </c>
       <c r="J5" t="n">
-        <v>399.8</v>
+        <v>131.47</v>
       </c>
       <c r="K5" t="n">
-        <v>387.1</v>
+        <v>130.54</v>
       </c>
       <c r="L5" t="n">
-        <v>394.89</v>
+        <v>131.87</v>
       </c>
       <c r="M5" t="n">
-        <v>371.53</v>
+        <v>127.87</v>
       </c>
       <c r="N5" t="n">
-        <v>426.81</v>
+        <v>137.34</v>
       </c>
       <c r="O5" t="n">
         <v>1.63</v>
@@ -925,17 +925,17 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>1.85</v>
+        <v>0</v>
       </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
-        <v>2.09</v>
+        <v>0</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="Y5" t="n">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -959,22 +959,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-12-TSLA</t>
+          <t>2026-05-14-V</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Autos / Tech</t>
+          <t>Pagos</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -992,26 +992,26 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>427.91</v>
+        <v>320.31</v>
       </c>
       <c r="J6" t="n">
-        <v>445.27</v>
+        <v>320.31</v>
       </c>
       <c r="K6" t="n">
-        <v>422.04</v>
+        <v>317.55</v>
       </c>
       <c r="L6" t="n">
-        <v>430.42</v>
+        <v>321.49</v>
       </c>
       <c r="M6" t="n">
-        <v>405.28</v>
+        <v>309.67</v>
       </c>
       <c r="N6" t="n">
-        <v>464.78</v>
+        <v>337.65</v>
       </c>
       <c r="O6" t="n">
         <v>1.63</v>
@@ -1027,56 +1027,56 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Y6" t="n">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAJO</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-12-SPY</t>
+          <t>2026-05-14-TEAM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ETF Mercado</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>734.6799999999999</v>
+        <v>80.62</v>
       </c>
       <c r="J7" t="n">
-        <v>742.3099999999999</v>
+        <v>80.62</v>
       </c>
       <c r="K7" t="n">
-        <v>732.3200000000001</v>
+        <v>78.31999999999999</v>
       </c>
       <c r="L7" t="n">
-        <v>735.6900000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>725.58</v>
+        <v>71.77</v>
       </c>
       <c r="N7" t="n">
-        <v>749.51</v>
+        <v>95.05</v>
       </c>
       <c r="O7" t="n">
         <v>1.63</v>
@@ -1129,56 +1129,56 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>1.04</v>
+        <v>0</v>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
-        <v>1.15</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Y7" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MEDIO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-12-SOXX</t>
+          <t>2026-05-14-SNOW</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ETF Chips</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1200,22 +1200,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>503.79</v>
+        <v>152.37</v>
       </c>
       <c r="J8" t="n">
-        <v>528.29</v>
+        <v>152.37</v>
       </c>
       <c r="K8" t="n">
-        <v>497.06</v>
+        <v>149.6</v>
       </c>
       <c r="L8" t="n">
-        <v>506.67</v>
+        <v>153.56</v>
       </c>
       <c r="M8" t="n">
-        <v>477.83</v>
+        <v>141.69</v>
       </c>
       <c r="N8" t="n">
-        <v>546.1</v>
+        <v>169.78</v>
       </c>
       <c r="O8" t="n">
         <v>1.63</v>
@@ -1231,56 +1231,56 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>4.86</v>
+        <v>0</v>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
-        <v>5.13</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>VIGILAR</t>
+          <t>POSIBLE COMPRA</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="Y8" t="n">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MEDIO</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-12-SLB</t>
+          <t>2026-05-14-SBUX</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>SBUX</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Energía</t>
+          <t>Consumo</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1294,30 +1294,30 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>55.68</v>
+        <v>105.95</v>
       </c>
       <c r="J9" t="n">
-        <v>55.38</v>
+        <v>105.95</v>
       </c>
       <c r="K9" t="n">
-        <v>55.11</v>
+        <v>104.96</v>
       </c>
       <c r="L9" t="n">
-        <v>55.92</v>
+        <v>106.38</v>
       </c>
       <c r="M9" t="n">
-        <v>53.49</v>
+        <v>102.11</v>
       </c>
       <c r="N9" t="n">
-        <v>59.25</v>
+        <v>112.2</v>
       </c>
       <c r="O9" t="n">
         <v>1.63</v>
@@ -1333,17 +1333,17 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>-0.54</v>
+        <v>0</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.54</v>
+        <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
@@ -1356,33 +1356,33 @@
         </is>
       </c>
       <c r="Y9" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-12-LRCX</t>
+          <t>2026-05-14-ORCL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Equipos chips</t>
+          <t>Tecnología</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1404,22 +1404,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>283.1</v>
+        <v>189.76</v>
       </c>
       <c r="J10" t="n">
-        <v>295.44</v>
+        <v>189.76</v>
       </c>
       <c r="K10" t="n">
-        <v>278.06</v>
+        <v>186.65</v>
       </c>
       <c r="L10" t="n">
-        <v>285.26</v>
+        <v>191.09</v>
       </c>
       <c r="M10" t="n">
-        <v>263.67</v>
+        <v>177.77</v>
       </c>
       <c r="N10" t="n">
-        <v>314.77</v>
+        <v>209.3</v>
       </c>
       <c r="O10" t="n">
         <v>1.63</v>
@@ -1435,17 +1435,17 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>4.36</v>
+        <v>0</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
-        <v>4.94</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
@@ -1458,33 +1458,33 @@
         </is>
       </c>
       <c r="Y10" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-12-KLAC</t>
+          <t>2026-05-14-OKTA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Equipos chips</t>
+          <t>Ciberseguridad</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1506,22 +1506,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1811.35</v>
+        <v>78.2</v>
       </c>
       <c r="J11" t="n">
-        <v>1849.71</v>
+        <v>78.2</v>
       </c>
       <c r="K11" t="n">
-        <v>1780.61</v>
+        <v>77.06999999999999</v>
       </c>
       <c r="L11" t="n">
-        <v>1824.53</v>
+        <v>78.68000000000001</v>
       </c>
       <c r="M11" t="n">
-        <v>1692.77</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>2004.59</v>
+        <v>85.28</v>
       </c>
       <c r="O11" t="n">
         <v>1.63</v>
@@ -1537,17 +1537,17 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>2.12</v>
+        <v>0</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="Y11" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -1571,22 +1571,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-12-COIN</t>
+          <t>2026-05-14-MS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COIN</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cripto / Trading</t>
+          <t>Finanzas</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1600,30 +1600,30 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>204.97</v>
+        <v>193.83</v>
       </c>
       <c r="J12" t="n">
-        <v>201.8</v>
+        <v>193.83</v>
       </c>
       <c r="K12" t="n">
-        <v>200.64</v>
+        <v>192.36</v>
       </c>
       <c r="L12" t="n">
-        <v>206.83</v>
+        <v>194.46</v>
       </c>
       <c r="M12" t="n">
-        <v>188.26</v>
+        <v>188.18</v>
       </c>
       <c r="N12" t="n">
-        <v>232.19</v>
+        <v>203.04</v>
       </c>
       <c r="O12" t="n">
         <v>1.63</v>
@@ -1639,17 +1639,17 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>-1.55</v>
+        <v>0</v>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.55</v>
+        <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
@@ -1662,33 +1662,33 @@
         </is>
       </c>
       <c r="Y12" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-12-AVGO</t>
+          <t>2026-05-14-MRVL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IA / Chips</t>
+          <t>Chips</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1702,30 +1702,30 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>415.2</v>
+        <v>177.95</v>
       </c>
       <c r="J13" t="n">
-        <v>416.79</v>
+        <v>177.95</v>
       </c>
       <c r="K13" t="n">
-        <v>409.81</v>
+        <v>174.19</v>
       </c>
       <c r="L13" t="n">
-        <v>417.51</v>
+        <v>179.56</v>
       </c>
       <c r="M13" t="n">
-        <v>394.42</v>
+        <v>163.45</v>
       </c>
       <c r="N13" t="n">
-        <v>449.06</v>
+        <v>201.59</v>
       </c>
       <c r="O13" t="n">
         <v>1.63</v>
@@ -1741,17 +1741,17 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>0.38</v>
+        <v>0</v>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
-        <v>0.99</v>
+        <v>0</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
@@ -1764,28 +1764,28 @@
         </is>
       </c>
       <c r="Y13" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-12-ASML</t>
+          <t>2026-05-14-MPWR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1812,22 +1812,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>1493.25</v>
+        <v>1650.35</v>
       </c>
       <c r="J14" t="n">
-        <v>1581.58</v>
+        <v>1650.35</v>
       </c>
       <c r="K14" t="n">
-        <v>1472</v>
+        <v>1622.63</v>
       </c>
       <c r="L14" t="n">
-        <v>1502.36</v>
+        <v>1662.23</v>
       </c>
       <c r="M14" t="n">
-        <v>1411.29</v>
+        <v>1543.44</v>
       </c>
       <c r="N14" t="n">
-        <v>1626.81</v>
+        <v>1824.57</v>
       </c>
       <c r="O14" t="n">
         <v>1.63</v>
@@ -1843,17 +1843,17 @@
         </is>
       </c>
       <c r="R14" t="n">
-        <v>5.92</v>
+        <v>0</v>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="n">
-        <v>5.92</v>
+        <v>0</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
@@ -1870,24 +1870,24 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-12-ARM</t>
+          <t>2026-05-14-MCHP</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MCHP</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1906,30 +1906,30 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>204.41</v>
+        <v>96.70999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>221.21</v>
+        <v>96.70999999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>198.08</v>
+        <v>95.16</v>
       </c>
       <c r="L15" t="n">
-        <v>207.12</v>
+        <v>97.38</v>
       </c>
       <c r="M15" t="n">
-        <v>179.98</v>
+        <v>90.72</v>
       </c>
       <c r="N15" t="n">
-        <v>244.22</v>
+        <v>106.48</v>
       </c>
       <c r="O15" t="n">
         <v>1.63</v>
@@ -1945,17 +1945,17 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>8.220000000000001</v>
+        <v>0</v>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="n">
-        <v>8.220000000000001</v>
+        <v>0</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
@@ -1968,33 +1968,33 @@
         </is>
       </c>
       <c r="Y15" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>MEDIO</t>
+          <t>BAJO</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-12-AMZN</t>
+          <t>2026-05-14-MARA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MARA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Tecnología</t>
+          <t>Cripto / Trading</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2008,30 +2008,30 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>264.04</v>
+        <v>12.75</v>
       </c>
       <c r="J16" t="n">
-        <v>270.13</v>
+        <v>12.75</v>
       </c>
       <c r="K16" t="n">
-        <v>261.5</v>
+        <v>12.43</v>
       </c>
       <c r="L16" t="n">
-        <v>265.13</v>
+        <v>12.89</v>
       </c>
       <c r="M16" t="n">
-        <v>254.24</v>
+        <v>11.5</v>
       </c>
       <c r="N16" t="n">
-        <v>280</v>
+        <v>14.79</v>
       </c>
       <c r="O16" t="n">
         <v>1.63</v>
@@ -2047,17 +2047,17 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="n">
-        <v>2.31</v>
+        <v>0</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
         </is>
       </c>
       <c r="Y16" t="n">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
@@ -2081,22 +2081,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-12-AMAT</t>
+          <t>2026-05-14-LLY</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Equipos chips</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2114,26 +2114,26 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>BAJO</t>
+          <t>MEDIO</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>421.22</v>
+        <v>1015.75</v>
       </c>
       <c r="J17" t="n">
-        <v>436.61</v>
+        <v>1015.75</v>
       </c>
       <c r="K17" t="n">
-        <v>414.6</v>
+        <v>1003.63</v>
       </c>
       <c r="L17" t="n">
-        <v>424.06</v>
+        <v>1020.95</v>
       </c>
       <c r="M17" t="n">
-        <v>395.69</v>
+        <v>968.99</v>
       </c>
       <c r="N17" t="n">
-        <v>462.82</v>
+        <v>1091.96</v>
       </c>
       <c r="O17" t="n">
         <v>1.63</v>
@@ -2149,17 +2149,17 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>3.65</v>
+        <v>0</v>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="n">
-        <v>3.71</v>
+        <v>0</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
@@ -2175,6 +2175,3270 @@
         <v>96</v>
       </c>
       <c r="Z17" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-14-JNJ</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>89</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>230.42</v>
+      </c>
+      <c r="J18" t="n">
+        <v>230.42</v>
+      </c>
+      <c r="K18" t="n">
+        <v>229.05</v>
+      </c>
+      <c r="L18" t="n">
+        <v>231.01</v>
+      </c>
+      <c r="M18" t="n">
+        <v>225.12</v>
+      </c>
+      <c r="N18" t="n">
+        <v>239.06</v>
+      </c>
+      <c r="O18" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y18" t="n">
+        <v>89</v>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-14-IWM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ETF Russell</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>85</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>282.67</v>
+      </c>
+      <c r="J19" t="n">
+        <v>282.67</v>
+      </c>
+      <c r="K19" t="n">
+        <v>281.16</v>
+      </c>
+      <c r="L19" t="n">
+        <v>283.32</v>
+      </c>
+      <c r="M19" t="n">
+        <v>276.84</v>
+      </c>
+      <c r="N19" t="n">
+        <v>292.17</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y19" t="n">
+        <v>85</v>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-14-HAL</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>96</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="J20" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="K20" t="n">
+        <v>40.62</v>
+      </c>
+      <c r="L20" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="M20" t="n">
+        <v>39.47</v>
+      </c>
+      <c r="N20" t="n">
+        <v>43.54</v>
+      </c>
+      <c r="O20" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y20" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-14-GS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GS</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Finanzas</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>BUY STRONG</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>96</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>955.42</v>
+      </c>
+      <c r="J21" t="n">
+        <v>955.42</v>
+      </c>
+      <c r="K21" t="n">
+        <v>947.62</v>
+      </c>
+      <c r="L21" t="n">
+        <v>958.76</v>
+      </c>
+      <c r="M21" t="n">
+        <v>925.3200000000001</v>
+      </c>
+      <c r="N21" t="n">
+        <v>1004.47</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>BUY STRONG</t>
+        </is>
+      </c>
+      <c r="Y21" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-14-FANG</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FANG</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>96</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>201.1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>201.1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>198.87</v>
+      </c>
+      <c r="L22" t="n">
+        <v>202.06</v>
+      </c>
+      <c r="M22" t="n">
+        <v>192.49</v>
+      </c>
+      <c r="N22" t="n">
+        <v>215.13</v>
+      </c>
+      <c r="O22" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y22" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-14-EOG</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EOG</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>75</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>134.93</v>
+      </c>
+      <c r="J23" t="n">
+        <v>134.93</v>
+      </c>
+      <c r="K23" t="n">
+        <v>133.67</v>
+      </c>
+      <c r="L23" t="n">
+        <v>135.47</v>
+      </c>
+      <c r="M23" t="n">
+        <v>130.06</v>
+      </c>
+      <c r="N23" t="n">
+        <v>142.86</v>
+      </c>
+      <c r="O23" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y23" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-14-DIA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DIA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ETF Dow</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>85</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>497.14</v>
+      </c>
+      <c r="J24" t="n">
+        <v>497.14</v>
+      </c>
+      <c r="K24" t="n">
+        <v>495.48</v>
+      </c>
+      <c r="L24" t="n">
+        <v>497.85</v>
+      </c>
+      <c r="M24" t="n">
+        <v>490.75</v>
+      </c>
+      <c r="N24" t="n">
+        <v>507.55</v>
+      </c>
+      <c r="O24" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y24" t="n">
+        <v>85</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-14-DELL</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>96</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>243.87</v>
+      </c>
+      <c r="J25" t="n">
+        <v>243.87</v>
+      </c>
+      <c r="K25" t="n">
+        <v>239.31</v>
+      </c>
+      <c r="L25" t="n">
+        <v>245.83</v>
+      </c>
+      <c r="M25" t="n">
+        <v>226.27</v>
+      </c>
+      <c r="N25" t="n">
+        <v>272.56</v>
+      </c>
+      <c r="O25" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y25" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-14-DE</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>74</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>580.65</v>
+      </c>
+      <c r="J26" t="n">
+        <v>580.65</v>
+      </c>
+      <c r="K26" t="n">
+        <v>575.0599999999999</v>
+      </c>
+      <c r="L26" t="n">
+        <v>583.04</v>
+      </c>
+      <c r="M26" t="n">
+        <v>559.1</v>
+      </c>
+      <c r="N26" t="n">
+        <v>615.77</v>
+      </c>
+      <c r="O26" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y26" t="n">
+        <v>74</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-14-COST</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>96</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>1033.08</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1033.08</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1026.02</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1036.1</v>
+      </c>
+      <c r="M27" t="n">
+        <v>1005.87</v>
+      </c>
+      <c r="N27" t="n">
+        <v>1077.43</v>
+      </c>
+      <c r="O27" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>0</v>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y27" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-14-CAT</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>96</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>902.3</v>
+      </c>
+      <c r="J28" t="n">
+        <v>902.3</v>
+      </c>
+      <c r="K28" t="n">
+        <v>891.73</v>
+      </c>
+      <c r="L28" t="n">
+        <v>906.83</v>
+      </c>
+      <c r="M28" t="n">
+        <v>861.52</v>
+      </c>
+      <c r="N28" t="n">
+        <v>968.76</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>0</v>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y28" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-14-BLK</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BLK</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Finanzas</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>BUY STRONG</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>96</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>1094.1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1094.1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1086.44</v>
+      </c>
+      <c r="L29" t="n">
+        <v>1097.38</v>
+      </c>
+      <c r="M29" t="n">
+        <v>1064.56</v>
+      </c>
+      <c r="N29" t="n">
+        <v>1142.24</v>
+      </c>
+      <c r="O29" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R29" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" t="n">
+        <v>0</v>
+      </c>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>BUY STRONG</t>
+        </is>
+      </c>
+      <c r="Y29" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-14-BA</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>BUY STRONG</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>96</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>240.6</v>
+      </c>
+      <c r="J30" t="n">
+        <v>240.6</v>
+      </c>
+      <c r="K30" t="n">
+        <v>238.41</v>
+      </c>
+      <c r="L30" t="n">
+        <v>241.54</v>
+      </c>
+      <c r="M30" t="n">
+        <v>232.14</v>
+      </c>
+      <c r="N30" t="n">
+        <v>254.39</v>
+      </c>
+      <c r="O30" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" t="n">
+        <v>0</v>
+      </c>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>BUY STRONG</t>
+        </is>
+      </c>
+      <c r="Y30" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-14-ADI</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ADI</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Chips</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>96</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>432.39</v>
+      </c>
+      <c r="J31" t="n">
+        <v>432.39</v>
+      </c>
+      <c r="K31" t="n">
+        <v>428.31</v>
+      </c>
+      <c r="L31" t="n">
+        <v>434.14</v>
+      </c>
+      <c r="M31" t="n">
+        <v>416.65</v>
+      </c>
+      <c r="N31" t="n">
+        <v>458.04</v>
+      </c>
+      <c r="O31" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R31" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y31" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-14-ACHR</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ACHR</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Movilidad aérea</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>85</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="J32" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="K32" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="L32" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="M32" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="N32" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="O32" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y32" t="n">
+        <v>85</v>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-14-ABBV</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>90</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>208.5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>208.5</v>
+      </c>
+      <c r="K33" t="n">
+        <v>206.51</v>
+      </c>
+      <c r="L33" t="n">
+        <v>209.35</v>
+      </c>
+      <c r="M33" t="n">
+        <v>200.84</v>
+      </c>
+      <c r="N33" t="n">
+        <v>220.98</v>
+      </c>
+      <c r="O33" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R33" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y33" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-13-SMCI</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Servidores IA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>74</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>32.21</v>
+      </c>
+      <c r="J34" t="n">
+        <v>32</v>
+      </c>
+      <c r="K34" t="n">
+        <v>31.41</v>
+      </c>
+      <c r="L34" t="n">
+        <v>32.55</v>
+      </c>
+      <c r="M34" t="n">
+        <v>29.11</v>
+      </c>
+      <c r="N34" t="n">
+        <v>37.26</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="V34" t="n">
+        <v>1</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y34" t="n">
+        <v>74</v>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-13-NVDA</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>IA / Chips</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>96</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>226.34</v>
+      </c>
+      <c r="J35" t="n">
+        <v>225.83</v>
+      </c>
+      <c r="K35" t="n">
+        <v>223.5</v>
+      </c>
+      <c r="L35" t="n">
+        <v>227.56</v>
+      </c>
+      <c r="M35" t="n">
+        <v>215.39</v>
+      </c>
+      <c r="N35" t="n">
+        <v>244.18</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="V35" t="n">
+        <v>1</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y35" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-12-XOM</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>75</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>150.85</v>
+      </c>
+      <c r="J36" t="n">
+        <v>151.57</v>
+      </c>
+      <c r="K36" t="n">
+        <v>149.44</v>
+      </c>
+      <c r="L36" t="n">
+        <v>151.45</v>
+      </c>
+      <c r="M36" t="n">
+        <v>145.42</v>
+      </c>
+      <c r="N36" t="n">
+        <v>159.7</v>
+      </c>
+      <c r="O36" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R36" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="U36" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="V36" t="n">
+        <v>2</v>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y36" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-12-TSM</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Chips</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>86</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>392.55</v>
+      </c>
+      <c r="J37" t="n">
+        <v>399.8</v>
+      </c>
+      <c r="K37" t="n">
+        <v>387.1</v>
+      </c>
+      <c r="L37" t="n">
+        <v>394.89</v>
+      </c>
+      <c r="M37" t="n">
+        <v>371.53</v>
+      </c>
+      <c r="N37" t="n">
+        <v>426.81</v>
+      </c>
+      <c r="O37" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" t="n">
+        <v>2</v>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y37" t="n">
+        <v>79</v>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-12-TSLA</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Autos / Tech</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>86</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>427.91</v>
+      </c>
+      <c r="J38" t="n">
+        <v>445.27</v>
+      </c>
+      <c r="K38" t="n">
+        <v>422.04</v>
+      </c>
+      <c r="L38" t="n">
+        <v>430.42</v>
+      </c>
+      <c r="M38" t="n">
+        <v>405.28</v>
+      </c>
+      <c r="N38" t="n">
+        <v>464.78</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R38" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" t="n">
+        <v>2</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>VIGILAR</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="Y38" t="n">
+        <v>59</v>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-12-SPY</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ETF Mercado</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>96</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>734.6799999999999</v>
+      </c>
+      <c r="J39" t="n">
+        <v>742.3099999999999</v>
+      </c>
+      <c r="K39" t="n">
+        <v>732.3200000000001</v>
+      </c>
+      <c r="L39" t="n">
+        <v>735.6900000000001</v>
+      </c>
+      <c r="M39" t="n">
+        <v>725.58</v>
+      </c>
+      <c r="N39" t="n">
+        <v>749.51</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R39" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
+        <v>2</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>VIGILAR</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="Y39" t="n">
+        <v>84</v>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-12-SOXX</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ETF Chips</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>96</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>503.79</v>
+      </c>
+      <c r="J40" t="n">
+        <v>528.29</v>
+      </c>
+      <c r="K40" t="n">
+        <v>497.06</v>
+      </c>
+      <c r="L40" t="n">
+        <v>506.67</v>
+      </c>
+      <c r="M40" t="n">
+        <v>477.83</v>
+      </c>
+      <c r="N40" t="n">
+        <v>546.1</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R40" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="n">
+        <v>2</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>VIGILAR</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="Y40" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-12-SLB</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SLB</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Energía</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>91</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>55.68</v>
+      </c>
+      <c r="J41" t="n">
+        <v>55.38</v>
+      </c>
+      <c r="K41" t="n">
+        <v>55.11</v>
+      </c>
+      <c r="L41" t="n">
+        <v>55.92</v>
+      </c>
+      <c r="M41" t="n">
+        <v>53.49</v>
+      </c>
+      <c r="N41" t="n">
+        <v>59.25</v>
+      </c>
+      <c r="O41" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R41" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="U41" t="n">
+        <v>-0.54</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2</v>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y41" t="n">
+        <v>92</v>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-12-LRCX</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Equipos chips</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>96</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>283.1</v>
+      </c>
+      <c r="J42" t="n">
+        <v>295.44</v>
+      </c>
+      <c r="K42" t="n">
+        <v>278.06</v>
+      </c>
+      <c r="L42" t="n">
+        <v>285.26</v>
+      </c>
+      <c r="M42" t="n">
+        <v>263.67</v>
+      </c>
+      <c r="N42" t="n">
+        <v>314.77</v>
+      </c>
+      <c r="O42" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R42" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2</v>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y42" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z42" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-12-KLAC</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Equipos chips</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>94</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>1811.35</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1849.71</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1780.61</v>
+      </c>
+      <c r="L43" t="n">
+        <v>1824.53</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1692.77</v>
+      </c>
+      <c r="N43" t="n">
+        <v>2004.59</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R43" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U43" t="n">
+        <v>0</v>
+      </c>
+      <c r="V43" t="n">
+        <v>2</v>
+      </c>
+      <c r="W43" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y43" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z43" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-12-COIN</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Cripto / Trading</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>87</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>204.97</v>
+      </c>
+      <c r="J44" t="n">
+        <v>201.8</v>
+      </c>
+      <c r="K44" t="n">
+        <v>200.64</v>
+      </c>
+      <c r="L44" t="n">
+        <v>206.83</v>
+      </c>
+      <c r="M44" t="n">
+        <v>188.26</v>
+      </c>
+      <c r="N44" t="n">
+        <v>232.19</v>
+      </c>
+      <c r="O44" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R44" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="U44" t="n">
+        <v>-1.55</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2</v>
+      </c>
+      <c r="W44" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y44" t="n">
+        <v>85</v>
+      </c>
+      <c r="Z44" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-12-AVGO</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>IA / Chips</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>74</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>415.2</v>
+      </c>
+      <c r="J45" t="n">
+        <v>416.79</v>
+      </c>
+      <c r="K45" t="n">
+        <v>409.81</v>
+      </c>
+      <c r="L45" t="n">
+        <v>417.51</v>
+      </c>
+      <c r="M45" t="n">
+        <v>394.42</v>
+      </c>
+      <c r="N45" t="n">
+        <v>449.06</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R45" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" t="n">
+        <v>2</v>
+      </c>
+      <c r="W45" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y45" t="n">
+        <v>86</v>
+      </c>
+      <c r="Z45" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-12-ASML</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Chips</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>96</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>1493.25</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1581.58</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1472</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1502.36</v>
+      </c>
+      <c r="M46" t="n">
+        <v>1411.29</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1626.81</v>
+      </c>
+      <c r="O46" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R46" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="U46" t="n">
+        <v>0</v>
+      </c>
+      <c r="V46" t="n">
+        <v>2</v>
+      </c>
+      <c r="W46" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X46" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y46" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z46" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-12-ARM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Chips</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>86</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>204.41</v>
+      </c>
+      <c r="J47" t="n">
+        <v>221.21</v>
+      </c>
+      <c r="K47" t="n">
+        <v>198.08</v>
+      </c>
+      <c r="L47" t="n">
+        <v>207.12</v>
+      </c>
+      <c r="M47" t="n">
+        <v>179.98</v>
+      </c>
+      <c r="N47" t="n">
+        <v>244.22</v>
+      </c>
+      <c r="O47" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R47" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="n">
+        <v>8.220000000000001</v>
+      </c>
+      <c r="U47" t="n">
+        <v>0</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2</v>
+      </c>
+      <c r="W47" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y47" t="n">
+        <v>84</v>
+      </c>
+      <c r="Z47" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-05-12-AMZN</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Tecnología</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>75</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>264.04</v>
+      </c>
+      <c r="J48" t="n">
+        <v>270.13</v>
+      </c>
+      <c r="K48" t="n">
+        <v>261.5</v>
+      </c>
+      <c r="L48" t="n">
+        <v>265.13</v>
+      </c>
+      <c r="M48" t="n">
+        <v>254.24</v>
+      </c>
+      <c r="N48" t="n">
+        <v>280</v>
+      </c>
+      <c r="O48" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R48" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="U48" t="n">
+        <v>0</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2</v>
+      </c>
+      <c r="W48" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X48" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y48" t="n">
+        <v>79</v>
+      </c>
+      <c r="Z48" t="inlineStr">
+        <is>
+          <t>MEDIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-05-12-AMAT</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Equipos chips</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>96</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>BAJO</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>421.22</v>
+      </c>
+      <c r="J49" t="n">
+        <v>436.61</v>
+      </c>
+      <c r="K49" t="n">
+        <v>414.6</v>
+      </c>
+      <c r="L49" t="n">
+        <v>424.06</v>
+      </c>
+      <c r="M49" t="n">
+        <v>395.69</v>
+      </c>
+      <c r="N49" t="n">
+        <v>462.82</v>
+      </c>
+      <c r="O49" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>ABIERTA</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>EN SEGUIMIENTO</t>
+        </is>
+      </c>
+      <c r="R49" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2</v>
+      </c>
+      <c r="W49" t="inlineStr">
+        <is>
+          <t>POSIBLE COMPRA</t>
+        </is>
+      </c>
+      <c r="X49" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="Y49" t="n">
+        <v>96</v>
+      </c>
+      <c r="Z49" t="inlineStr">
         <is>
           <t>MEDIO</t>
         </is>

</xml_diff>